<commit_message>
ready audit and chat wise ticket created
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,10 +476,8 @@
           <t>04-09-2026 14:34:41</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>916307343181</t>
-        </is>
+      <c r="B4" t="n">
+        <v>916307343181</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -487,6 +485,24 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>05-09-2026 10:03:28</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hdhx</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ready For whatsapp through created ticket  audio wise chat wise server proper response
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,17 +492,33 @@
           <t>05-09-2026 10:03:28</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hdhx</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05-09-2026 19:28:57</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>918140021166</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Hdhx</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>nbm</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
pending audio file attachement
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,10 +508,8 @@
           <t>05-09-2026 19:28:57</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>918140021166</t>
-        </is>
+      <c r="B6" t="n">
+        <v>918140021166</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -519,6 +517,262 @@
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>07-09-2026 11:32:44</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>07-09-2026 11:34:13</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07-09-2026 11:34:21</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>07-09-2026 11:45:31</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>919427950801</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07-09-2026 11:59:25</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:00:08</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Gemini API Error: [WinError 10054] An existing connection was forcibly closed by the remote host</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-2963465301391255.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:00:43</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>{'subject': 'Software is ready', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-37198685357629924.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:00:53</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Software is ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:02:03</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:33:57</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:35:53</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>{'subject': 'UPS not working properly', 'custom_issue_regarding': 'Hardware Support', 'remainder_date': '', 'priority': 'Medium', 'from_number': '916307343181'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:36:10</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Ticket inserted: UPS not working properly</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:36:27</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:37:13</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>{'subject': 'System RAM not working', 'custom_issue_regarding': 'Hardware Support', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\916307343181.mp3'}</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-08738753829453627.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>07-09-2026 12:37:24</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Ticket inserted: System RAM not working</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>07-09-2026 13:09:43</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>919310002625</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Audio FIle Insert And Assinger user send audio link ticket mode Done
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -764,14 +764,652 @@
           <t>07-09-2026 13:09:43</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>919310002625</t>
-        </is>
+      <c r="B22" t="n">
+        <v>919310002625</v>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:23:59</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:25:22</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>919327228987</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:29:25</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>919327228987</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:30:45</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>919327228987</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing Purpose', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'from_number': '919327228987'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:30:55</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>919327228987</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing Purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:47:39</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:49:18</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>{'subject': 'Just testing purpose this ticket is create', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-5612968796120413.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:49:27</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Just testing purpose this ticket is create</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:51:49</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:52:57</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-6723935861826089.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:58:14</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:59:05</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-9304887706859711.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08-09-2026 10:59:21</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:02:58</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:03:42</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-11360767485164247.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:03:56</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:04:49</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:07:30</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>919883690727</v>
+      </c>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:10:20</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:11:03</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>{'subject': 'Test ticket for testing purpose', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8190118978360351.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:11:25</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Test ticket for testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:12:44</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:13:31</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing ticket', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-3360795764588056.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:13:52</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:16:49</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:17:44</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-7023508261406172.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:18:04</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:19:39</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:20:22</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>919920248390</v>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:20:24</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-7122161283487078.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:20:43</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:20:48</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>919920248390</v>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:20:51</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>919920248390</v>
+      </c>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:21:37</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:22:16</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>{'subject': 'Po issues', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Medium', 'from_number': '916307343181'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:22:28</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Po issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:22:43</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:23:34</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>{'subject': 'UPI issue', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\916307343181.mp3'}</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-9854236250085353.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:23:54</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>916307343181</v>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Ticket inserted: UPI issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:34:47</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Produlation Ready Onlt Ticket Menu
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1402,13 +1402,423 @@
           <t>08-09-2026 11:34:47</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>918140021166</t>
-        </is>
+      <c r="B62" t="n">
+        <v>918140021166</v>
       </c>
       <c r="C62" t="inlineStr"/>
-      <c r="D62" t="b">
+      <c r="D62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:44:41</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:45:35</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>{'subject': 'Chatbot is ready to use in production', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-3322713906435423.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:45:58</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Chatbot is ready to use in production</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:48:14</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>919327228987</v>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:55:37</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>919726166466</v>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>08-09-2026 11:55:59</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>919726166466</v>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:07:53</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:08:34</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>{'subject': 'Inquiry about incoming viscose satin stock', 'custom_issue_regarding': 'SUBHASH SIR PAPAJI', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:08:41</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Inquiry about incoming viscose satin stock</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:11:47</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>919328213004</v>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:12:16</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:12:27</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>919328213004</v>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>{'subject': 'complete mill work urgently', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'High', 'from_number': '919328213004'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:12:37</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>919328213004</v>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Ticket inserted: complete mill work urgently</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:12:55</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:13:25</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose', 'custom_issue_regarding': 'SUBHASH SIR PAPAJI', 'remainder_date': '', 'priority': 'Low', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:13:31</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>{'subject': 'Finish the work urgently', 'custom_issue_regarding': 'SUBHASH SIR PAPAJI', 'remainder_date': '', 'priority': 'High', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:13:34</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:13:41</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Finish the work urgently</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:15:32</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>919328213004</v>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:16:09</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>919328213004</v>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>{'subject': 'testing this ticket system', 'custom_issue_regarding': 'Harsh Sir Raja bhaiya', 'remainder_date': '', 'priority': 'Low', 'from_number': '919328213004'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:16:22</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>919328213004</v>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Ticket inserted: testing this ticket system</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:26:11</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:30:24</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:31:31</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>{'subject': 'Car check this issues', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:32:31</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Car check this issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:36:22</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>918347089999</v>
+      </c>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:54:41</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Jobwork Order Add Endpont
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1812,14 +1812,590 @@
           <t>08-09-2026 12:54:41</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>918347089999</t>
-        </is>
+      <c r="B89" t="n">
+        <v>918347089999</v>
       </c>
       <c r="C89" t="inlineStr"/>
-      <c r="D89" t="b">
-        <v>1</v>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>08-09-2026 12:57:03</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:12:13</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:12:57</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>{'subject': 'Mention Kunal, meet Dinesh', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-13351709217005592.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:13:19</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>918140021166</v>
+      </c>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Mention Kunal, meet Dinesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:48:22</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:49:04</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:51:05</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:51:26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:52:27</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:54:20</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:54:40</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:55:32</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:55:49</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:56:30</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:56:45</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:57:32</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>08-09-2026 14:57:57</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:00:38</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:06:24</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>919327228987</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:07:03</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>919327228987</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:07:17</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:11:26</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>919327228987</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:11:42</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:14:10</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:15:32</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>{custom.number_check}</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:17:46</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:25:25</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>919327228987</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:32:39</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>{recipient.mobileNo}</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:35:09</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:36:07</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:36:42</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:39:27</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:40:32</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>919327228987</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>08-09-2026 15:41:14</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>919327228987</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
self Ticket View  Done
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D253"/>
+  <dimension ref="A1:D257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4648,6 +4648,70 @@
         </is>
       </c>
     </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>11-09-2026 19:43:05</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr"/>
+      <c r="D254" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>11-09-2026 19:44:28</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr"/>
+      <c r="D255" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>11-09-2026 20:03:17</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr"/>
+      <c r="D256" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>11-09-2026 20:06:57</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr"/>
+      <c r="D257" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
assign Ticket View Done
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D260"/>
+  <dimension ref="A1:D262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4756,7 +4756,39 @@
         </is>
       </c>
       <c r="C260" t="inlineStr"/>
-      <c r="D260" t="b">
+      <c r="D260" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>11-09-2026 21:04:00</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr"/>
+      <c r="D261" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>11-09-2026 21:06:41</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr"/>
+      <c r="D262" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Url assigned_a_ticket This Funcation Had issue Fix URL Link  issue
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D262"/>
+  <dimension ref="A1:D355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4788,8 +4788,1690 @@
         </is>
       </c>
       <c r="C262" t="inlineStr"/>
-      <c r="D262" t="b">
-        <v>1</v>
+      <c r="D262" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>12-09-2026 09:49:35</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr"/>
+      <c r="D263" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>12-09-2026 09:50:50</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr"/>
+      <c r="D264" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:07:57</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr"/>
+      <c r="D265" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:09:40</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>917203005550</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr"/>
+      <c r="D266" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:12:36</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>917203005550</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr"/>
+      <c r="D267" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:13:06</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>917203005550</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr"/>
+      <c r="D268" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:27:29</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr"/>
+      <c r="D269" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:29:28</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr"/>
+      <c r="D270" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:30:12</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr"/>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>{'subject': 'testing purpose', 'custom_issue_regarding': 'rahul patil', 'remainder_date': '', 'priority': '', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:30:22</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr"/>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Ticket inserted: testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:35:57</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr"/>
+      <c r="D273" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:36:34</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr"/>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>{'subject': 'testing purpose', 'custom_issue_regarding': 'rahul patil', 'remainder_date': '', 'priority': 'Low', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:36:44</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr"/>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Ticket inserted: testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:58:23</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>919974972625</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr"/>
+      <c r="D276" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>12-09-2026 11:59:14</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>919974972625</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr"/>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>12-09-2026 12:18:06</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr"/>
+      <c r="D278" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>12-09-2026 12:35:39</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr"/>
+      <c r="D279" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>12-09-2026 12:38:00</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr"/>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>{'subject': 'PO error', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Medium', 'from_number': '916307343181'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>12-09-2026 12:38:23</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr"/>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Ticket inserted: PO error</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:18:20</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr"/>
+      <c r="D282" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:19:17</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>{'subject': 'GR report update and tasar silk stock update', 'custom_issue_regarding': 'Jai Shankar Ji', 'remainder_date': '2026-09-14', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-1714956859136132.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:19:33</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr"/>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Ticket inserted: GR report update and tasar silk stock update</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:20:30</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr"/>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:21:19</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>{'subject': 'Accounts related ticket', 'custom_issue_regarding': 'himanshu', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-9836685386405459.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:21:39</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr"/>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Accounts related ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:22:43</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr"/>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:23:42</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>{'subject': 'Finalize embroidery machine installation in front building', 'custom_issue_regarding': 'Harsh Sir Raja bhaiya', 'remainder_date': '2026-09-14', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-7541154604852697.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:23:59</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr"/>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Finalize embroidery machine installation in front building</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:25:49</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>{'subject': 'Update on Sunil Morchhari production report', 'custom_issue_regarding': 'Rakesh Panday RFD', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-4138929547964242.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:26:07</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr"/>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Update on Sunil Morchhari production report</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:27:49</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr"/>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Audio URL: Hi</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:30:38</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr"/>
+      <c r="D294" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:31:17</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing ticket', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8264922085691797.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:31:41</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr"/>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:35:04</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr"/>
+      <c r="D297" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:37:06</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>{'subject': 'Test testing purpose 1 number ticket create', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': '', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-2625649221942389.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:37:29</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr"/>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Test testing purpose 1 number ticket create</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:38:45</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr"/>
+      <c r="D300" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:57:00</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr"/>
+      <c r="D301" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:58:41</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr"/>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Audio URL: Hey</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:59:01</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing 1 2 3', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-6122063065842027.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>12-09-2026 13:59:17</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr"/>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing 1 2 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:10:00</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr"/>
+      <c r="D305" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:10:42</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>{'subject': 'testing 123', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-15490206220645397.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:10:58</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr"/>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Ticket inserted: testing 123</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:14:06</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr"/>
+      <c r="D308" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:14:40</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing 1 2 3', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-6730447063631594.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:14:56</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr"/>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing 1 2 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:25:03</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr"/>
+      <c r="D311" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:25:52</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-2543071362825372.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:26:22</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr"/>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:26:54</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose 2', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-3023378761884916.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:27:08</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr"/>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:37:20</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr"/>
+      <c r="D316" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:41:16</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr"/>
+      <c r="D317" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:42:59</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr"/>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '919558856235'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:44:38</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr"/>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:45:03</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr"/>
+      <c r="D320" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:45:34</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr"/>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>{'subject': 'Po issues', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Medium', 'from_number': '916307343181'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>12-09-2026 14:45:43</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr"/>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Po issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:01:44</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr"/>
+      <c r="D323" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:03:19</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr"/>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>{'subject': '200 Days above The Shokin Customer Payment Not received', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'High', 'from_number': '919558856235'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:03:35</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>919558856235</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr"/>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Ticket inserted: 200 Days above The Shokin Customer Payment Not received</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:04:18</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr"/>
+      <c r="D326" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:05:18</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>{'subject': 'Pending staff salary issue', 'custom_issue_regarding': 'Hiren Account', 'remainder_date': '', 'priority': 'High', 'audio_path': 'audio_file\\919081833391.mp3'}</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8126622303520984.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:05:37</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr"/>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Pending staff salary issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:06:36</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>{'subject': 'Ask Pathak ji for response', 'custom_issue_regarding': 'Dipak Ca Pathak', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\919081833391.mp3'}</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-9756558330630591.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:06:38</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr"/>
+      <c r="D330" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:07:09</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr"/>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Ask Pathak ji for response</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:08:15</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>{'subject': 'Reply needed for ticket 00257 regarding staff salary', 'custom_issue_regarding': 'Hiren Account', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\919081833391.mp3'}</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8254265133489473.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:08:40</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr"/>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Reply needed for ticket 00257 regarding staff salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:09:22</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>{'subject': 'Staff salary pending date', 'custom_issue_regarding': 'Hiren Account', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\919081833391.mp3'}</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-823139521007994.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:09:41</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>919081833391</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr"/>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Staff salary pending date</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:18:50</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr"/>
+      <c r="D336" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:20:14</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr"/>
+      <c r="D337" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:21:12</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>{'subject': 'Software issue', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\916307343181.mp3'}</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-4561876836177339.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>12-09-2026 15:21:51</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr"/>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Software issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:01:14</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr"/>
+      <c r="D340" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:01:49</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr"/>
+      <c r="D341" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:02:15</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>{'subject': 'Change PPT in chatbot menu image', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-24358305054551943.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:02:25</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr"/>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>{'subject': 'Keep a track on harbans dupatta sent to mill', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:02:36</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr"/>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Change PPT in chatbot menu image</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:03:53</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr"/>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:04:24</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr"/>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:05:09</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>{'subject': 'Harbans dupatta mill reminder', 'custom_issue_regarding': '', 'remainder_date': '2026-09-14', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-6367065525991464.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:05:25</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr"/>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Harbans dupatta mill reminder</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:07:56</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr"/>
+      <c r="D349" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:19:34</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr"/>
+      <c r="D350" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:20:11</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>{'subject': 'Change PPT in chatbot menu image', 'custom_issue_regarding': 'ateesh', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-03370752872706628.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:56:31</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr"/>
+      <c r="D352" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:57:13</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr"/>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>{'subject': 'Gokul Chatbot Number', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:57:23</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr"/>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Gokul Chatbot Number</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>12-09-2026 16:58:28</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>919830553100</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr"/>
+      <c r="D355" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Feauter Add For Dicet Voice Or Chat Message After Direct Ticket Created Main Menu By pass
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D355"/>
+  <dimension ref="A1:D371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6474,6 +6474,284 @@
         <v>0</v>
       </c>
     </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>12-09-2026 17:11:37</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>916307343181</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr"/>
+      <c r="D356" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:10:48</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr"/>
+      <c r="D357" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:11:18</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr"/>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:11:26</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr"/>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:13:34</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr"/>
+      <c r="D360" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:13:59</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr"/>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:14:05</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>919920248390</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr"/>
+      <c r="D362" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:14:21</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr"/>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:14:28</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr"/>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:16:08</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr"/>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:16:16</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr"/>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:23:13</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr"/>
+      <c r="D367" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:23:59</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket create', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-3852876138210436.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>12-09-2026 19:24:14</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr"/>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket create</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>12-09-2026 20:36:37</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>919379783261</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr"/>
+      <c r="D370" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>12-09-2026 21:58:14</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr"/>
+      <c r="D371" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
number add backup purpose commit
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D371"/>
+  <dimension ref="A1:D421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6748,7 +6748,871 @@
         </is>
       </c>
       <c r="C371" t="inlineStr"/>
-      <c r="D371" t="b">
+      <c r="D371" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>21-09-2026 11:24:04</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr"/>
+      <c r="D372" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>21-09-2026 11:27:51</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr"/>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>{'subject': 'Check Rap Linen ultra pei sampling status', 'custom_issue_regarding': 'SUBHASH SIR PAPAJI', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>21-09-2026 11:28:01</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr"/>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Check Rap Linen ultra pei sampling status</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>21-09-2026 11:44:04</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr"/>
+      <c r="D375" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>21-09-2026 11:45:16</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>{'subject': 'Salesman wise sale report after every tour', 'custom_issue_regarding': 'Dipak Ca Pathak', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8295479373665904.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>21-09-2026 11:45:39</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr"/>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Salesman wise sale report after every tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:14:56</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr"/>
+      <c r="D378" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:16:25</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr"/>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>{'subject': 'Create salesman wise report with fabric status to track progress of each salesman', 'custom_issue_regarding': 'Rakesh Panday RFD', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:16:35</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr"/>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Create salesman wise report with fabric status to track progress of each salesman</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:17:36</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr"/>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>{'subject': 'Rakesh pandey need to take proper decision for the fabrics coming gr from sachin', 'custom_issue_regarding': 'Rakesh Panday RFD', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:17:46</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr"/>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Rakesh pandey need to take proper decision for the fabrics coming gr from sachin</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:22:03</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr"/>
+      <c r="D383" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:24:55</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr"/>
+      <c r="D384" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:26:06</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr"/>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>{'subject': 'Keep track for gaji duppatta as we have to sell this season', 'custom_issue_regarding': 'Chandan Print Salesman', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:27:49</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr"/>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Keep track for gaji duppatta as we have to sell this season</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:34:01</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr"/>
+      <c r="D387" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:46:24</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr"/>
+      <c r="D388" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:47:40</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr"/>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>{'subject': 'check this new ticket system', 'custom_issue_regarding': 'Kunal Embdyed', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:47:58</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr"/>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Ticket inserted: check this new ticket system</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:52:33</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>919375373663</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr"/>
+      <c r="D391" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:53:29</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>919375373663</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr"/>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>{'subject': 'final rate for gajji dupatta', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'Medium', 'from_number': '919375373663'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:56:01</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr"/>
+      <c r="D393" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>21-09-2026 12:56:35</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>919328865295</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr"/>
+      <c r="D394" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>21-09-2026 13:43:01</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr"/>
+      <c r="D395" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>21-09-2026 13:46:48</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr"/>
+      <c r="D396" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>21-09-2026 13:49:39</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr"/>
+      <c r="D397" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>21-09-2026 13:49:48</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr"/>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>{'subject': 'Raven in cutting done but not delivered challan EMBDYED warehouse transfer issue update', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>21-09-2026 13:50:25</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr"/>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Raven in cutting done but not delivered challan EMBDYED warehouse transfer issue update</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:10:34</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr"/>
+      <c r="D400" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:16:01</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr"/>
+      <c r="D401" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:21:40</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr"/>
+      <c r="D402" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:28:43</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr"/>
+      <c r="D403" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:28:57</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr"/>
+      <c r="D404" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:30:27</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr"/>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>{'subject': 'Raven in cutting done but not delivered challan EMBDYED warehouse transfer issue', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:30:56</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr"/>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Raven in cutting done but not delivered challan EMBDYED warehouse transfer issue</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:31:58</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr"/>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-05086707935281909.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:32:42</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr"/>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8060972231981309.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:35:47</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr"/>
+      <c r="D409" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:36:03</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr"/>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>{'subject': 'Raven in cutting done but not delivered challan EMBDYED warehouse transfer issue update', 'custom_issue_regarding': 'Siddharth Sir', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:36:11</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr"/>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Raven in cutting done but not delivered challan EMBDYED warehouse transfer issue update</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:36:52</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>{'subject': 'Testing purpose ticket create', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-48018253685237167.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>21-09-2026 14:37:10</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr"/>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Testing purpose ticket create</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>21-09-2026 15:15:59</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>917203030140</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr"/>
+      <c r="D414" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>21-09-2026 15:25:11</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr"/>
+      <c r="D415" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>21-09-2026 17:17:57</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>919328865295</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr"/>
+      <c r="D416" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>21-09-2026 17:18:21</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>919737250004</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr"/>
+      <c r="D417" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>21-09-2026 17:18:56</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>919328865295</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr"/>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>21-09-2026 17:19:50</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>919328865295</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>{'subject': 'Radhika export kali development update pending', 'custom_issue_regarding': 'Harsh Sir Raja bhaiya', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\919328865295.mp3'}</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-2836520267520223.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>21-09-2026 17:20:12</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>919328865295</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr"/>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Radhika export kali development update pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>21-09-2026 17:27:30</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>919328905446</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr"/>
+      <c r="D421" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Feauter For Auto Remainder Ticket
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D421"/>
+  <dimension ref="A1:D424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7612,8 +7612,56 @@
         </is>
       </c>
       <c r="C421" t="inlineStr"/>
-      <c r="D421" t="b">
-        <v>1</v>
+      <c r="D421" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>21-09-2026 18:40:27</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>917838300240</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr"/>
+      <c r="D422" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>21-09-2026 19:23:36</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>919821228796</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr"/>
+      <c r="D423" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>21-09-2026 19:23:47</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>919821228796</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr"/>
+      <c r="D424" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update after some issue fix
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D424"/>
+  <dimension ref="A1:D426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7664,6 +7664,40 @@
         <v>0</v>
       </c>
     </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>27-09-2026 14:34:13</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr"/>
+      <c r="D425" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>27-09-2026 14:36:34</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr"/>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Producation server backup purpose
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D426"/>
+  <dimension ref="A1:D438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7698,6 +7698,214 @@
         </is>
       </c>
     </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>27-09-2026 15:11:51</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr"/>
+      <c r="D427" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>27-09-2026 15:40:05</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr"/>
+      <c r="D428" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>27-09-2026 15:41:10</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr"/>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>27-09-2026 15:42:16</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr"/>
+      <c r="D430" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>27-09-2026 15:44:31</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr"/>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>28-09-2026 08:34:17</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr"/>
+      <c r="D432" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>28-09-2026 08:34:38</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr"/>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/undefined</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>28-09-2026 08:35:11</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>{'subject': 'Lift ka quotation finalization', 'custom_issue_regarding': 'HR Laxminarayan Sharma', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-7938912732247757.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>28-09-2026 08:35:40</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr"/>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Lift ka quotation finalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>28-09-2026 10:19:33</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>919737250002</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr"/>
+      <c r="D436" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>28-09-2026 10:20:19</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr"/>
+      <c r="D437" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>28-09-2026 10:22:14</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>919737250002</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr"/>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Ticket inserted: None</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Some Report Issue Fix
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D438"/>
+  <dimension ref="A1:D467"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7906,6 +7906,522 @@
         </is>
       </c>
     </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>29-09-2026 10:37:34</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr"/>
+      <c r="D439" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:22:28</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr"/>
+      <c r="D440" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:22:58</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>{'subject': 'Check payment for South Cotton', 'custom_issue_regarding': 'Prakash Karn Account', 'remainder_date': '', 'priority': 'High', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-8693706233518792.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:23:20</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr"/>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Check payment for South Cotton</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:24:13</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>918511832625</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr"/>
+      <c r="D443" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:25:43</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr"/>
+      <c r="D444" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:26:12</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>{'subject': 'Maal Rajshri mein bhej ke RFD karwana hai aur Papaji ko update karna hai', 'custom_issue_regarding': 'Tej Bahadur Grey', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-12156910447636449.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:26:14</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>918511832625</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr"/>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>{'subject': 'Fan removed from EMBDYED section not reinstalled', 'custom_issue_regarding': 'HR Laxminarayan Sharma', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918511832625'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:26:28</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr"/>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Maal Rajshri mein bhej ke RFD karwana hai aur Papaji ko update karna hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:26:43</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>918511832625</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr"/>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Fan removed from EMBDYED section not reinstalled</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:27:07</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>{'subject': 'Send material to Rajshree and update Papaji', 'custom_issue_regarding': 'Tej Bahadur Grey', 'remainder_date': '', 'priority': 'Medium', 'audio_path': 'audio_file\\918347089999.mp3'}</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-0719315855742233.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:27:19</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr"/>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Send material to Rajshree and update Papaji</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:29:26</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr"/>
+      <c r="D451" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:30:26</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr"/>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>{'subject': 'Need a report as to how many tickets we raise to hns', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:31:09</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr"/>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>{'subject': 'Need a report on how many tickets we raise to hns dinesh', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '', 'priority': 'Low', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:34:53</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>918140661069</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr"/>
+      <c r="D454" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:47:23</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr"/>
+      <c r="D455" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:48:02</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr"/>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>{'subject': 'Inform HODs to keep action points ready for Saturday meeting', 'custom_issue_regarding': 'HR Laxminarayan Sharma', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918347089999'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:48:18</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>918347089999</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr"/>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Inform HODs to keep action points ready for Saturday meeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:52:59</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr"/>
+      <c r="D458" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:56:05</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr"/>
+      <c r="D459" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:56:21</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr"/>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>{'subject': 'hello testing', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>29-09-2026 11:59:31</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>{'subject': '', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': '', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-72587542259708.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>29-09-2026 12:00:06</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>{'subject': 'Ticket for testing purpose', 'custom_issue_regarding': '', 'remainder_date': '', 'priority': 'Low', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-6310050512525658.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>29-09-2026 12:08:31</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr"/>
+      <c r="D463" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>29-09-2026 12:09:35</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr"/>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>{'subject': 'Send message in English', 'custom_issue_regarding': 'Paulmi madam', 'remainder_date': '', 'priority': 'Medium', 'from_number': '918140021166'}</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>29-09-2026 18:19:14</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr"/>
+      <c r="D465" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>29-09-2026 18:20:13</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr"/>
+      <c r="D466" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>29-09-2026 18:21:50</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr"/>
+      <c r="D467" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Producation ready Server waitress Add For Help Server Safe to Crack
</commit_message>
<xml_diff>
--- a/log.xlsx
+++ b/log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D486"/>
+  <dimension ref="A1:D492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8736,8 +8736,118 @@
         </is>
       </c>
       <c r="C486" t="inlineStr"/>
-      <c r="D486" t="b">
-        <v>1</v>
+      <c r="D486" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>01-10-2026 19:16:15</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr"/>
+      <c r="D487" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>01-10-2026 19:16:38</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr"/>
+      <c r="D488" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>01-10-2026 19:20:32</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr"/>
+      <c r="D489" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>01-10-2026 19:21:45</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>{'subject': 'Camera and Wifi problem', 'custom_issue_regarding': 'Dinesh Software', 'remainder_date': '2026-10-02', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-4176296590188394.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>01-10-2026 19:22:41</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>{'subject': 'Camera and WiFi issue in PNH company', 'custom_issue_regarding': 'Hardware Support', 'remainder_date': '2026-10-02', 'priority': 'Medium', 'audio_path': 'audio_file\\918140021166.mp3'}</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Audio URL: https://11zamedia.11za.in/gokultexprintsprivatelimited/Receive/AUD/AUD-37664458349512264.ogg</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>01-10-2026 19:23:15</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>918140021166</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr"/>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Ticket inserted: Camera and WiFi issue in PNH company</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>